<commit_message>
chore(preview): nouveaux outputs AAPL post-corrections (pdf+pptx+xlsx)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/preview/AAPL/AAPL_financials.xlsx
+++ b/preview/AAPL/AAPL_financials.xlsx
@@ -9429,7 +9429,7 @@
       <c r="F95" s="266" t="n"/>
       <c r="G95" s="266" t="n"/>
       <c r="H95" s="266" t="n">
-        <v>253.38</v>
+        <v>253.68</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -9555,7 +9555,7 @@
       <c r="F100" s="266" t="n"/>
       <c r="G100" s="266" t="n"/>
       <c r="H100" s="266" t="n">
-        <v>0.0433</v>
+        <v>0.0432</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -9623,7 +9623,7 @@
       <c r="F103" s="266" t="n"/>
       <c r="G103" s="266" t="n"/>
       <c r="H103" s="266" t="n">
-        <v>0.0583</v>
+        <v>0.0582</v>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
@@ -10001,10 +10001,7 @@
       <c r="A123" s="3" t="n"/>
       <c r="B123" s="14" t="n"/>
       <c r="C123" s="3" t="n"/>
-      <c r="D123" s="22">
-        <f>== SYNTHESE IA ===</f>
-        <v/>
-      </c>
+      <c r="D123" s="22" t="n"/>
       <c r="E123" s="22" t="n"/>
       <c r="F123" s="22" t="n"/>
       <c r="G123" s="22" t="n"/>
@@ -10018,11 +10015,7 @@
         </is>
       </c>
       <c r="C124" s="2" t="n"/>
-      <c r="D124" s="25" t="inlineStr">
-        <is>
-          <t>Recommandation : BUY</t>
-        </is>
-      </c>
+      <c r="D124" s="25" t="n"/>
       <c r="E124" s="25" t="n"/>
       <c r="F124" s="25" t="n"/>
       <c r="G124" s="25" t="n"/>
@@ -10036,11 +10029,7 @@
         </is>
       </c>
       <c r="C125" s="2" t="n"/>
-      <c r="D125" s="25" t="inlineStr">
-        <is>
-          <t>Conviction     : 80%</t>
-        </is>
-      </c>
+      <c r="D125" s="25" t="n"/>
       <c r="E125" s="25" t="n"/>
       <c r="F125" s="25" t="n"/>
       <c r="G125" s="25" t="n"/>
@@ -10054,11 +10043,7 @@
         </is>
       </c>
       <c r="C126" s="2" t="n"/>
-      <c r="D126" s="25" t="inlineStr">
-        <is>
-          <t>Confiance IA   : 80%</t>
-        </is>
-      </c>
+      <c r="D126" s="25" t="n"/>
       <c r="E126" s="25" t="n"/>
       <c r="F126" s="25" t="n"/>
       <c r="G126" s="25" t="n"/>
@@ -10066,20 +10051,14 @@
     </row>
     <row r="127" ht="15" customHeight="1">
       <c r="B127" s="51" t="n"/>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>Cible Base : 280.5</t>
-        </is>
-      </c>
     </row>
     <row r="128" ht="3" customHeight="1">
       <c r="A128" s="417" t="n"/>
       <c r="B128" s="418" t="n"/>
       <c r="C128" s="417" t="n"/>
-      <c r="D128" s="419" t="inlineStr">
-        <is>
-          <t>Cible Bull : 310.2</t>
-        </is>
+      <c r="D128" s="419">
+        <f>IF(COUNTA(D9,D10,D14,D15,D16,D20,D21,D25)=8,1,0)+IF(COUNTA(E9,E10,E14,E15,E16,E20,E21,E25)=8,1,0)+IF(COUNTA(F9,F10,F14,F15,F16,F20,F21,F25)=8,1,0)+IF(COUNTA(G9,G10,G14,G15,G16,G20,G21,G25)=8,1,0)</f>
+        <v/>
       </c>
       <c r="E128" s="419" t="n"/>
       <c r="F128" s="419">
@@ -10097,27 +10076,12 @@
     </row>
     <row r="129" ht="15" customHeight="1">
       <c r="B129" s="51" t="n"/>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>Cible Bear : 240.8</t>
-        </is>
-      </c>
     </row>
     <row r="130" ht="15" customHeight="1">
       <c r="B130" s="51" t="n"/>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>Apple Inc. presente une opportunité d'investissement attractive avec des perspectives de croissance solides et une position dominante sur le marché. L'entreprise devrait poursuivre sa croissance grâce</t>
-        </is>
-      </c>
     </row>
     <row r="131" ht="15" customHeight="1">
       <c r="B131" s="51" t="n"/>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>Invalidation : Récession économique mondiale, concurrence accrue dans le secteur des smartphones, problèmes de production ou de livraison</t>
-        </is>
-      </c>
     </row>
     <row r="132" ht="15" customHeight="1">
       <c r="B132" s="51" t="n"/>
@@ -10410,7 +10374,7 @@
         </is>
       </c>
       <c r="C14" s="536" t="n">
-        <v>253.35</v>
+        <v>253.68</v>
       </c>
     </row>
     <row r="15">
@@ -20305,7 +20269,7 @@
         </is>
       </c>
       <c r="D9" s="477" t="n">
-        <v>374</v>
+        <v>370.36</v>
       </c>
       <c r="E9" s="36" t="n">
         <v>2801644.86</v>
@@ -20346,7 +20310,7 @@
         </is>
       </c>
       <c r="D10" s="477" t="n">
-        <v>291.89</v>
+        <v>288.45</v>
       </c>
       <c r="E10" s="36" t="n">
         <v>3438605.5</v>
@@ -20387,7 +20351,7 @@
         </is>
       </c>
       <c r="D11" s="477" t="n">
-        <v>599.8200000000001</v>
+        <v>597.96</v>
       </c>
       <c r="E11" s="36" t="n">
         <v>1503313</v>
@@ -20428,7 +20392,7 @@
         </is>
       </c>
       <c r="D12" s="477" t="n">
-        <v>20.68</v>
+        <v>20.59</v>
       </c>
       <c r="E12" s="36" t="n">
         <v>49113.28</v>

</xml_diff>

<commit_message>
chore(preview): AAPL outputs post-corrections PDF v3 (market cap, football field, P9 methodologie)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/preview/AAPL/AAPL_financials.xlsx
+++ b/preview/AAPL/AAPL_financials.xlsx
@@ -9429,7 +9429,7 @@
       <c r="F95" s="266" t="n"/>
       <c r="G95" s="266" t="n"/>
       <c r="H95" s="266" t="n">
-        <v>253.68</v>
+        <v>253.53</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -10001,7 +10001,11 @@
       <c r="A123" s="3" t="n"/>
       <c r="B123" s="14" t="n"/>
       <c r="C123" s="3" t="n"/>
-      <c r="D123" s="22" t="n"/>
+      <c r="D123" s="22" t="inlineStr">
+        <is>
+          <t>--- SYNTHESE IA ---</t>
+        </is>
+      </c>
       <c r="E123" s="22" t="n"/>
       <c r="F123" s="22" t="n"/>
       <c r="G123" s="22" t="n"/>
@@ -10015,7 +10019,11 @@
         </is>
       </c>
       <c r="C124" s="2" t="n"/>
-      <c r="D124" s="25" t="n"/>
+      <c r="D124" s="25" t="inlineStr">
+        <is>
+          <t>Recommandation : BUY</t>
+        </is>
+      </c>
       <c r="E124" s="25" t="n"/>
       <c r="F124" s="25" t="n"/>
       <c r="G124" s="25" t="n"/>
@@ -10029,7 +10037,11 @@
         </is>
       </c>
       <c r="C125" s="2" t="n"/>
-      <c r="D125" s="25" t="n"/>
+      <c r="D125" s="25" t="inlineStr">
+        <is>
+          <t>Conviction : 80%</t>
+        </is>
+      </c>
       <c r="E125" s="25" t="n"/>
       <c r="F125" s="25" t="n"/>
       <c r="G125" s="25" t="n"/>
@@ -10043,7 +10055,11 @@
         </is>
       </c>
       <c r="C126" s="2" t="n"/>
-      <c r="D126" s="25" t="n"/>
+      <c r="D126" s="25" t="inlineStr">
+        <is>
+          <t>Confiance IA : 80%</t>
+        </is>
+      </c>
       <c r="E126" s="25" t="n"/>
       <c r="F126" s="25" t="n"/>
       <c r="G126" s="25" t="n"/>
@@ -10051,6 +10067,11 @@
     </row>
     <row r="127" ht="15" customHeight="1">
       <c r="B127" s="51" t="n"/>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Cible Base : 270.0</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="3" customHeight="1">
       <c r="A128" s="417" t="n"/>
@@ -10076,12 +10097,27 @@
     </row>
     <row r="129" ht="15" customHeight="1">
       <c r="B129" s="51" t="n"/>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Cible Bear : 230.0</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="15" customHeight="1">
       <c r="B130" s="51" t="n"/>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Apple Inc. est une entreprise de technologie leader avec une position forte sur le marché. La croissance des revenus et des marges est attendue.</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="15" customHeight="1">
       <c r="B131" s="51" t="n"/>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Invalidation : Récession économique, concurrence accrue dans le secteur des smartphones, problèmes de production d'iPhones</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="15" customHeight="1">
       <c r="B132" s="51" t="n"/>
@@ -10374,7 +10410,7 @@
         </is>
       </c>
       <c r="C14" s="536" t="n">
-        <v>253.68</v>
+        <v>253.53</v>
       </c>
     </row>
     <row r="15">
@@ -20269,7 +20305,7 @@
         </is>
       </c>
       <c r="D9" s="477" t="n">
-        <v>370.36</v>
+        <v>370.44</v>
       </c>
       <c r="E9" s="36" t="n">
         <v>2801644.86</v>
@@ -20310,7 +20346,7 @@
         </is>
       </c>
       <c r="D10" s="477" t="n">
-        <v>288.45</v>
+        <v>289.08</v>
       </c>
       <c r="E10" s="36" t="n">
         <v>3438605.5</v>
@@ -20351,7 +20387,7 @@
         </is>
       </c>
       <c r="D11" s="477" t="n">
-        <v>597.96</v>
+        <v>598.36</v>
       </c>
       <c r="E11" s="36" t="n">
         <v>1503313</v>

</xml_diff>

<commit_message>
chore(preview): AAPL outputs mis a jour (slide2 risk body fix)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/preview/AAPL/AAPL_financials.xlsx
+++ b/preview/AAPL/AAPL_financials.xlsx
@@ -9429,7 +9429,7 @@
       <c r="F95" s="266" t="n"/>
       <c r="G95" s="266" t="n"/>
       <c r="H95" s="266" t="n">
-        <v>253.53</v>
+        <v>253.38</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -9555,7 +9555,7 @@
       <c r="F100" s="266" t="n"/>
       <c r="G100" s="266" t="n"/>
       <c r="H100" s="266" t="n">
-        <v>0.0432</v>
+        <v>0.0433</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -9623,7 +9623,7 @@
       <c r="F103" s="266" t="n"/>
       <c r="G103" s="266" t="n"/>
       <c r="H103" s="266" t="n">
-        <v>0.0582</v>
+        <v>0.0583</v>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
@@ -10001,10 +10001,9 @@
       <c r="A123" s="3" t="n"/>
       <c r="B123" s="14" t="n"/>
       <c r="C123" s="3" t="n"/>
-      <c r="D123" s="22" t="inlineStr">
-        <is>
-          <t>--- SYNTHESE IA ---</t>
-        </is>
+      <c r="D123" s="22">
+        <f>== SYNTHESE IA ===</f>
+        <v/>
       </c>
       <c r="E123" s="22" t="n"/>
       <c r="F123" s="22" t="n"/>
@@ -10039,7 +10038,7 @@
       <c r="C125" s="2" t="n"/>
       <c r="D125" s="25" t="inlineStr">
         <is>
-          <t>Conviction : 80%</t>
+          <t>Conviction     : 80%</t>
         </is>
       </c>
       <c r="E125" s="25" t="n"/>
@@ -10057,7 +10056,7 @@
       <c r="C126" s="2" t="n"/>
       <c r="D126" s="25" t="inlineStr">
         <is>
-          <t>Confiance IA : 80%</t>
+          <t>Confiance IA   : 80%</t>
         </is>
       </c>
       <c r="E126" s="25" t="n"/>
@@ -10069,7 +10068,7 @@
       <c r="B127" s="51" t="n"/>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Cible Base : 270.0</t>
+          <t>Cible Base : 280.5</t>
         </is>
       </c>
     </row>
@@ -10077,9 +10076,10 @@
       <c r="A128" s="417" t="n"/>
       <c r="B128" s="418" t="n"/>
       <c r="C128" s="417" t="n"/>
-      <c r="D128" s="419">
-        <f>IF(COUNTA(D9,D10,D14,D15,D16,D20,D21,D25)=8,1,0)+IF(COUNTA(E9,E10,E14,E15,E16,E20,E21,E25)=8,1,0)+IF(COUNTA(F9,F10,F14,F15,F16,F20,F21,F25)=8,1,0)+IF(COUNTA(G9,G10,G14,G15,G16,G20,G21,G25)=8,1,0)</f>
-        <v/>
+      <c r="D128" s="419" t="inlineStr">
+        <is>
+          <t>Cible Bull : 310.2</t>
+        </is>
       </c>
       <c r="E128" s="419" t="n"/>
       <c r="F128" s="419">
@@ -10099,7 +10099,7 @@
       <c r="B129" s="51" t="n"/>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Cible Bear : 230.0</t>
+          <t>Cible Bear : 240.8</t>
         </is>
       </c>
     </row>
@@ -10107,7 +10107,7 @@
       <c r="B130" s="51" t="n"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Apple Inc. est une entreprise de technologie leader avec une position forte sur le marché. La croissance des revenus et des marges est attendue.</t>
+          <t>Apple Inc. presente une opportunité d'investissement attractive avec des perspectives de croissance solides et une position dominante sur le marché. L'entreprise devrait poursuivre sa croissance grâce</t>
         </is>
       </c>
     </row>
@@ -10115,7 +10115,7 @@
       <c r="B131" s="51" t="n"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Invalidation : Récession économique, concurrence accrue dans le secteur des smartphones, problèmes de production d'iPhones</t>
+          <t>Invalidation : Récession économique mondiale, concurrence accrue dans le secteur des smartphones, problèmes de production ou de livraison</t>
         </is>
       </c>
     </row>
@@ -10410,7 +10410,7 @@
         </is>
       </c>
       <c r="C14" s="536" t="n">
-        <v>253.53</v>
+        <v>253.35</v>
       </c>
     </row>
     <row r="15">
@@ -20305,7 +20305,7 @@
         </is>
       </c>
       <c r="D9" s="477" t="n">
-        <v>370.44</v>
+        <v>374</v>
       </c>
       <c r="E9" s="36" t="n">
         <v>2801644.86</v>
@@ -20346,7 +20346,7 @@
         </is>
       </c>
       <c r="D10" s="477" t="n">
-        <v>289.08</v>
+        <v>291.89</v>
       </c>
       <c r="E10" s="36" t="n">
         <v>3438605.5</v>
@@ -20387,7 +20387,7 @@
         </is>
       </c>
       <c r="D11" s="477" t="n">
-        <v>598.36</v>
+        <v>599.8200000000001</v>
       </c>
       <c r="E11" s="36" t="n">
         <v>1503313</v>
@@ -20428,7 +20428,7 @@
         </is>
       </c>
       <c r="D12" s="477" t="n">
-        <v>20.59</v>
+        <v>20.68</v>
       </c>
       <c r="E12" s="36" t="n">
         <v>49113.28</v>

</xml_diff>

<commit_message>
fix(pdf): EBITDA unite incorrecte — supprimer heuristique 50k dans _frm + previews AAPL/TSLA/MSFT
Correction : _frm() divisait par 1000 seulement si valeur > 50 000, laissant
l'EBITDA TSLA (17 657M = 17,7Md$) s'afficher comme '17 657' au lieu de '17,7'.
Toutes les valeurs sont en millions (yfinance + LLM prompt) — toujours diviser par 1000.

Previews regeneres avec tous les correctifs PDF de la session :
- AAPL : nouveau format (Points cles, vigilance, graphiques remplis)
- TSLA : synthese BUY conviction=0.8, EBITDA en Md$ corriges
- MSFT : mise a jour livrables

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/preview/AAPL/AAPL_financials.xlsx
+++ b/preview/AAPL/AAPL_financials.xlsx
@@ -7600,19 +7600,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D9" s="266" t="n"/>
+      <c r="D9" s="266" t="n">
+        <v>394328</v>
+      </c>
       <c r="E9" s="266" t="n">
-        <v>394328</v>
+        <v>383285</v>
       </c>
       <c r="F9" s="266" t="n">
-        <v>383285</v>
+        <v>391035</v>
       </c>
       <c r="G9" s="266" t="n">
-        <v>391035</v>
-      </c>
-      <c r="H9" s="266" t="n">
         <v>416161</v>
       </c>
+      <c r="H9" s="266" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="3" t="n"/>
@@ -7626,19 +7626,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D10" s="267" t="n"/>
+      <c r="D10" s="267" t="n">
+        <v>-223546</v>
+      </c>
       <c r="E10" s="267" t="n">
-        <v>-223546</v>
+        <v>-214137</v>
       </c>
       <c r="F10" s="267" t="n">
-        <v>-214137</v>
+        <v>-210352</v>
       </c>
       <c r="G10" s="267" t="n">
-        <v>-210352</v>
-      </c>
-      <c r="H10" s="267" t="n">
         <v>-220960</v>
       </c>
+      <c r="H10" s="267" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="3" t="n"/>
@@ -7720,19 +7720,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D14" s="266" t="n"/>
+      <c r="D14" s="266" t="n">
+        <v>-25094</v>
+      </c>
       <c r="E14" s="266" t="n">
-        <v>-25094</v>
+        <v>-24932</v>
       </c>
       <c r="F14" s="266" t="n">
-        <v>-24932</v>
+        <v>-26097</v>
       </c>
       <c r="G14" s="266" t="n">
-        <v>-26097</v>
-      </c>
-      <c r="H14" s="266" t="n">
         <v>-27601</v>
       </c>
+      <c r="H14" s="266" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="3" t="n"/>
@@ -7746,19 +7746,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D15" s="266" t="n"/>
+      <c r="D15" s="266" t="n">
+        <v>-26251</v>
+      </c>
       <c r="E15" s="266" t="n">
-        <v>-26251</v>
+        <v>-29915</v>
       </c>
       <c r="F15" s="266" t="n">
-        <v>-29915</v>
+        <v>-31370</v>
       </c>
       <c r="G15" s="266" t="n">
-        <v>-31370</v>
-      </c>
-      <c r="H15" s="266" t="n">
         <v>-34550</v>
       </c>
+      <c r="H15" s="266" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="3" t="n"/>
@@ -7772,19 +7772,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D16" s="268" t="n"/>
+      <c r="D16" s="268" t="n">
+        <v>-11104</v>
+      </c>
       <c r="E16" s="268" t="n">
-        <v>-11104</v>
+        <v>-11519</v>
       </c>
       <c r="F16" s="268" t="n">
-        <v>-11519</v>
+        <v>-11445</v>
       </c>
       <c r="G16" s="268" t="n">
-        <v>-11445</v>
-      </c>
-      <c r="H16" s="268" t="n">
         <v>-11698</v>
       </c>
+      <c r="H16" s="268" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="3" t="n"/>
@@ -7867,15 +7867,17 @@
         </is>
       </c>
       <c r="D20" s="266" t="n">
-        <v>-2645</v>
+        <v>-2931</v>
       </c>
       <c r="E20" s="266" t="n">
-        <v>-2931</v>
+        <v>-3933</v>
       </c>
       <c r="F20" s="266" t="n">
-        <v>-3933</v>
-      </c>
-      <c r="G20" s="266" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="266" t="n">
+        <v>0</v>
+      </c>
       <c r="H20" s="266" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -7891,15 +7893,17 @@
         </is>
       </c>
       <c r="D21" s="268" t="n">
-        <v>2843</v>
+        <v>2825</v>
       </c>
       <c r="E21" s="268" t="n">
-        <v>2825</v>
+        <v>3750</v>
       </c>
       <c r="F21" s="268" t="n">
-        <v>3750</v>
-      </c>
-      <c r="G21" s="268" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G21" s="268" t="n">
+        <v>0</v>
+      </c>
       <c r="H21" s="268" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -7982,19 +7986,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D25" s="266" t="n"/>
+      <c r="D25" s="266" t="n">
+        <v>-19300</v>
+      </c>
       <c r="E25" s="266" t="n">
-        <v>-19300</v>
+        <v>-16741</v>
       </c>
       <c r="F25" s="266" t="n">
-        <v>-16741</v>
+        <v>-29749</v>
       </c>
       <c r="G25" s="266" t="n">
-        <v>-29749</v>
-      </c>
-      <c r="H25" s="266" t="n">
         <v>-20719</v>
       </c>
+      <c r="H25" s="266" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" thickBot="1">
       <c r="A26" s="3" t="n"/>
@@ -8145,19 +8149,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D34" s="269" t="n"/>
+      <c r="D34" s="269" t="n">
+        <v>23646</v>
+      </c>
       <c r="E34" s="269" t="n">
-        <v>23646</v>
+        <v>29965</v>
       </c>
       <c r="F34" s="269" t="n">
-        <v>29965</v>
+        <v>29943</v>
       </c>
       <c r="G34" s="269" t="n">
-        <v>29943</v>
-      </c>
-      <c r="H34" s="269" t="n">
         <v>35934</v>
       </c>
+      <c r="H34" s="269" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="3" t="n"/>
@@ -8171,19 +8175,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D35" s="266" t="n"/>
+      <c r="D35" s="266" t="n">
+        <v>28184</v>
+      </c>
       <c r="E35" s="266" t="n">
-        <v>28184</v>
+        <v>29508</v>
       </c>
       <c r="F35" s="266" t="n">
-        <v>29508</v>
+        <v>33410</v>
       </c>
       <c r="G35" s="266" t="n">
-        <v>33410</v>
-      </c>
-      <c r="H35" s="266" t="n">
         <v>39777</v>
       </c>
+      <c r="H35" s="266" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="3" t="n"/>
@@ -8197,19 +8201,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D36" s="266" t="n"/>
+      <c r="D36" s="266" t="n">
+        <v>4946</v>
+      </c>
       <c r="E36" s="266" t="n">
-        <v>4946</v>
+        <v>6331</v>
       </c>
       <c r="F36" s="266" t="n">
-        <v>6331</v>
+        <v>7286</v>
       </c>
       <c r="G36" s="266" t="n">
-        <v>7286</v>
-      </c>
-      <c r="H36" s="266" t="n">
         <v>5718</v>
       </c>
+      <c r="H36" s="266" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="3" t="n"/>
@@ -8223,19 +8227,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D37" s="268" t="n"/>
+      <c r="D37" s="268" t="n">
+        <v>21223</v>
+      </c>
       <c r="E37" s="268" t="n">
-        <v>21223</v>
+        <v>14695</v>
       </c>
       <c r="F37" s="268" t="n">
-        <v>14695</v>
+        <v>14287</v>
       </c>
       <c r="G37" s="268" t="n">
-        <v>14287</v>
-      </c>
-      <c r="H37" s="268" t="n">
         <v>14585</v>
       </c>
+      <c r="H37" s="268" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="3" t="n"/>
@@ -8302,19 +8306,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D41" s="266" t="n"/>
+      <c r="D41" s="266" t="n">
+        <v>42117</v>
+      </c>
       <c r="E41" s="266" t="n">
-        <v>42117</v>
+        <v>43715</v>
       </c>
       <c r="F41" s="266" t="n">
-        <v>43715</v>
+        <v>45680</v>
       </c>
       <c r="G41" s="266" t="n">
-        <v>45680</v>
-      </c>
-      <c r="H41" s="266" t="n">
         <v>49834</v>
       </c>
+      <c r="H41" s="266" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="3" t="n"/>
@@ -8346,19 +8350,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D43" s="266" t="n"/>
+      <c r="D43" s="266" t="n">
+        <v>39053</v>
+      </c>
       <c r="E43" s="266" t="n">
-        <v>39053</v>
+        <v>46906</v>
       </c>
       <c r="F43" s="266" t="n">
-        <v>46906</v>
+        <v>55335</v>
       </c>
       <c r="G43" s="266" t="n">
-        <v>55335</v>
-      </c>
-      <c r="H43" s="266" t="n">
         <v>62950</v>
       </c>
+      <c r="H43" s="266" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
       <c r="A44" s="3" t="n"/>
@@ -8425,19 +8429,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D47" s="266" t="n"/>
+      <c r="D47" s="266" t="n">
+        <v>64115</v>
+      </c>
       <c r="E47" s="266" t="n">
-        <v>64115</v>
+        <v>62611</v>
       </c>
       <c r="F47" s="266" t="n">
-        <v>62611</v>
+        <v>68960</v>
       </c>
       <c r="G47" s="266" t="n">
-        <v>68960</v>
-      </c>
-      <c r="H47" s="266" t="n">
         <v>69860</v>
       </c>
+      <c r="H47" s="266" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="3" t="n"/>
@@ -8451,19 +8455,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D48" s="266" t="n"/>
+      <c r="D48" s="266" t="n">
+        <v>21110</v>
+      </c>
       <c r="E48" s="266" t="n">
-        <v>21110</v>
+        <v>15807</v>
       </c>
       <c r="F48" s="266" t="n">
-        <v>15807</v>
+        <v>20879</v>
       </c>
       <c r="G48" s="266" t="n">
-        <v>20879</v>
-      </c>
-      <c r="H48" s="266" t="n">
         <v>20329</v>
       </c>
+      <c r="H48" s="266" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="3" t="n"/>
@@ -8477,19 +8481,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D49" s="266" t="n"/>
+      <c r="D49" s="266" t="n">
+        <v>6552</v>
+      </c>
       <c r="E49" s="266" t="n">
-        <v>6552</v>
+        <v>8819</v>
       </c>
       <c r="F49" s="266" t="n">
-        <v>8819</v>
+        <v>26601</v>
       </c>
       <c r="G49" s="266" t="n">
-        <v>26601</v>
-      </c>
-      <c r="H49" s="266" t="n">
         <v>13016</v>
       </c>
+      <c r="H49" s="266" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="3" t="n"/>
@@ -8503,19 +8507,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D50" s="268" t="n"/>
+      <c r="D50" s="268" t="n">
+        <v>52630</v>
+      </c>
       <c r="E50" s="268" t="n">
-        <v>52630</v>
+        <v>50010</v>
       </c>
       <c r="F50" s="268" t="n">
-        <v>50010</v>
+        <v>44024</v>
       </c>
       <c r="G50" s="268" t="n">
-        <v>44024</v>
-      </c>
-      <c r="H50" s="268" t="n">
         <v>44452</v>
       </c>
+      <c r="H50" s="268" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="3" t="n"/>
@@ -8582,19 +8586,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D54" s="268" t="n"/>
+      <c r="D54" s="268" t="n">
+        <v>98959</v>
+      </c>
       <c r="E54" s="268" t="n">
-        <v>98959</v>
+        <v>95281</v>
       </c>
       <c r="F54" s="268" t="n">
-        <v>95281</v>
+        <v>85750</v>
       </c>
       <c r="G54" s="268" t="n">
-        <v>85750</v>
-      </c>
-      <c r="H54" s="268" t="n">
         <v>78328</v>
       </c>
+      <c r="H54" s="268" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="3" t="n"/>
@@ -8661,19 +8665,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D58" s="266" t="n"/>
+      <c r="D58" s="266" t="n">
+        <v>64849</v>
+      </c>
       <c r="E58" s="266" t="n">
-        <v>64849</v>
+        <v>73812</v>
       </c>
       <c r="F58" s="266" t="n">
-        <v>73812</v>
+        <v>83276</v>
       </c>
       <c r="G58" s="266" t="n">
-        <v>83276</v>
-      </c>
-      <c r="H58" s="266" t="n">
         <v>93568</v>
       </c>
+      <c r="H58" s="266" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="3" t="n"/>
@@ -8911,19 +8915,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D71" s="266" t="n"/>
+      <c r="D71" s="266" t="n">
+        <v>-9343</v>
+      </c>
       <c r="E71" s="266" t="n">
-        <v>-9343</v>
+        <v>-417</v>
       </c>
       <c r="F71" s="266" t="n">
-        <v>-417</v>
+        <v>-5144</v>
       </c>
       <c r="G71" s="266" t="n">
-        <v>-5144</v>
-      </c>
-      <c r="H71" s="266" t="n">
         <v>-7029</v>
       </c>
+      <c r="H71" s="266" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="3" t="n"/>
@@ -8937,19 +8941,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D72" s="266" t="n"/>
+      <c r="D72" s="266" t="n">
+        <v>1484</v>
+      </c>
       <c r="E72" s="266" t="n">
-        <v>1484</v>
+        <v>-1618</v>
       </c>
       <c r="F72" s="266" t="n">
-        <v>-1618</v>
+        <v>-1046</v>
       </c>
       <c r="G72" s="266" t="n">
-        <v>-1046</v>
-      </c>
-      <c r="H72" s="266" t="n">
         <v>1400</v>
       </c>
+      <c r="H72" s="266" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="3" t="n"/>
@@ -8963,19 +8967,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D73" s="266" t="n"/>
+      <c r="D73" s="266" t="n">
+        <v>9448</v>
+      </c>
       <c r="E73" s="266" t="n">
-        <v>9448</v>
+        <v>-1889</v>
       </c>
       <c r="F73" s="266" t="n">
-        <v>-1889</v>
+        <v>6020</v>
       </c>
       <c r="G73" s="266" t="n">
-        <v>6020</v>
-      </c>
-      <c r="H73" s="266" t="n">
         <v>902</v>
       </c>
+      <c r="H73" s="266" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="3" t="n"/>
@@ -8989,19 +8993,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D74" s="266" t="n"/>
+      <c r="D74" s="266" t="n">
+        <v>1006</v>
+      </c>
       <c r="E74" s="266" t="n">
-        <v>1006</v>
+        <v>-2227</v>
       </c>
       <c r="F74" s="266" t="n">
-        <v>-2227</v>
+        <v>-2266</v>
       </c>
       <c r="G74" s="266" t="n">
-        <v>-2266</v>
-      </c>
-      <c r="H74" s="266" t="n">
         <v>-89</v>
       </c>
+      <c r="H74" s="266" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" thickBot="1">
       <c r="A75" s="3" t="n"/>
@@ -9068,19 +9072,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D78" s="266" t="n"/>
+      <c r="D78" s="266" t="n">
+        <v>-10708</v>
+      </c>
       <c r="E78" s="266" t="n">
-        <v>-10708</v>
+        <v>-10959</v>
       </c>
       <c r="F78" s="266" t="n">
-        <v>-10959</v>
+        <v>-9447</v>
       </c>
       <c r="G78" s="266" t="n">
-        <v>-9447</v>
-      </c>
-      <c r="H78" s="266" t="n">
         <v>-12715</v>
       </c>
+      <c r="H78" s="266" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="3" t="n"/>
@@ -9165,19 +9169,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D83" s="266" t="n"/>
+      <c r="D83" s="266" t="n">
+        <v>5465</v>
+      </c>
       <c r="E83" s="266" t="n">
-        <v>5465</v>
+        <v>5228</v>
       </c>
       <c r="F83" s="266" t="n">
-        <v>5228</v>
+        <v>0</v>
       </c>
       <c r="G83" s="266" t="n">
-        <v>0</v>
-      </c>
-      <c r="H83" s="266" t="n">
         <v>4481</v>
       </c>
+      <c r="H83" s="266" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="3" t="n"/>
@@ -9192,20 +9196,18 @@
         </is>
       </c>
       <c r="D84" s="266" t="n">
-        <v>1105</v>
+        <v>-89402</v>
       </c>
       <c r="E84" s="266" t="n">
-        <v>-89402</v>
+        <v>-77550</v>
       </c>
       <c r="F84" s="266" t="n">
-        <v>-77550</v>
+        <v>-94949</v>
       </c>
       <c r="G84" s="266" t="n">
-        <v>-94949</v>
-      </c>
-      <c r="H84" s="266" t="n">
         <v>-90711</v>
       </c>
+      <c r="H84" s="266" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="3" t="n"/>
@@ -9219,19 +9221,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D85" s="266" t="n"/>
+      <c r="D85" s="266" t="n">
+        <v>-89402</v>
+      </c>
       <c r="E85" s="266" t="n">
-        <v>-89402</v>
+        <v>-77550</v>
       </c>
       <c r="F85" s="266" t="n">
-        <v>-77550</v>
+        <v>-94949</v>
       </c>
       <c r="G85" s="266" t="n">
-        <v>-94949</v>
-      </c>
-      <c r="H85" s="266" t="n">
         <v>-90711</v>
       </c>
+      <c r="H85" s="266" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1" thickBot="1">
       <c r="A86" s="3" t="n"/>
@@ -9331,19 +9333,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D90" s="266" t="n"/>
+      <c r="D90" s="266" t="n">
+        <v>35929</v>
+      </c>
       <c r="E90" s="266" t="n">
-        <v>35929</v>
+        <v>24977</v>
       </c>
       <c r="F90" s="266" t="n">
-        <v>24977</v>
+        <v>30737</v>
       </c>
       <c r="G90" s="266" t="n">
-        <v>30737</v>
-      </c>
-      <c r="H90" s="266" t="n">
         <v>29943</v>
       </c>
+      <c r="H90" s="266" t="n"/>
     </row>
     <row r="91" ht="15" customHeight="1" thickBot="1">
       <c r="A91" s="3" t="n"/>
@@ -9429,7 +9431,7 @@
       <c r="F95" s="266" t="n"/>
       <c r="G95" s="266" t="n"/>
       <c r="H95" s="266" t="n">
-        <v>253.38</v>
+        <v>254.2</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -9555,7 +9557,7 @@
       <c r="F100" s="266" t="n"/>
       <c r="G100" s="266" t="n"/>
       <c r="H100" s="266" t="n">
-        <v>0.0433</v>
+        <v>0.0432</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -9623,7 +9625,7 @@
       <c r="F103" s="266" t="n"/>
       <c r="G103" s="266" t="n"/>
       <c r="H103" s="266" t="n">
-        <v>0.0583</v>
+        <v>0.0582</v>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
@@ -10001,9 +10003,10 @@
       <c r="A123" s="3" t="n"/>
       <c r="B123" s="14" t="n"/>
       <c r="C123" s="3" t="n"/>
-      <c r="D123" s="22">
-        <f>== SYNTHESE IA ===</f>
-        <v/>
+      <c r="D123" s="22" t="inlineStr">
+        <is>
+          <t>--- SYNTHESE IA ---</t>
+        </is>
       </c>
       <c r="E123" s="22" t="n"/>
       <c r="F123" s="22" t="n"/>
@@ -10038,7 +10041,7 @@
       <c r="C125" s="2" t="n"/>
       <c r="D125" s="25" t="inlineStr">
         <is>
-          <t>Conviction     : 80%</t>
+          <t>Conviction : 78%</t>
         </is>
       </c>
       <c r="E125" s="25" t="n"/>
@@ -10056,7 +10059,7 @@
       <c r="C126" s="2" t="n"/>
       <c r="D126" s="25" t="inlineStr">
         <is>
-          <t>Confiance IA   : 80%</t>
+          <t>Confiance IA : 82%</t>
         </is>
       </c>
       <c r="E126" s="25" t="n"/>
@@ -10068,7 +10071,7 @@
       <c r="B127" s="51" t="n"/>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Cible Base : 280.5</t>
+          <t>Cible Base : 285.0</t>
         </is>
       </c>
     </row>
@@ -10076,10 +10079,9 @@
       <c r="A128" s="417" t="n"/>
       <c r="B128" s="418" t="n"/>
       <c r="C128" s="417" t="n"/>
-      <c r="D128" s="419" t="inlineStr">
-        <is>
-          <t>Cible Bull : 310.2</t>
-        </is>
+      <c r="D128" s="419">
+        <f>IF(COUNTA(D9,D10,D14,D15,D16,D20,D21,D25)=8,1,0)+IF(COUNTA(E9,E10,E14,E15,E16,E20,E21,E25)=8,1,0)+IF(COUNTA(F9,F10,F14,F15,F16,F20,F21,F25)=8,1,0)+IF(COUNTA(G9,G10,G14,G15,G16,G20,G21,G25)=8,1,0)</f>
+        <v/>
       </c>
       <c r="E128" s="419" t="n"/>
       <c r="F128" s="419">
@@ -10099,7 +10101,7 @@
       <c r="B129" s="51" t="n"/>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Cible Bear : 240.8</t>
+          <t>Cible Bear : 240.0</t>
         </is>
       </c>
     </row>
@@ -10107,7 +10109,7 @@
       <c r="B130" s="51" t="n"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Apple Inc. presente une opportunité d'investissement attractive avec des perspectives de croissance solides et une position dominante sur le marché. L'entreprise devrait poursuivre sa croissance grâce</t>
+          <t>Apple maintient une position dominante dans les services et l'innovation hardware malgré des défis macroéconomiques. La valorisation reste attractive avec une marge nette de 26.9% et un ROIC de 84.4%.</t>
         </is>
       </c>
     </row>
@@ -10115,7 +10117,7 @@
       <c r="B131" s="51" t="n"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Invalidation : Récession économique mondiale, concurrence accrue dans le secteur des smartphones, problèmes de production ou de livraison</t>
+          <t>Invalidation : Régulation App Store, récession mondiale ou échec iPhone 17</t>
         </is>
       </c>
     </row>
@@ -10410,7 +10412,7 @@
         </is>
       </c>
       <c r="C14" s="536" t="n">
-        <v>253.35</v>
+        <v>254.2</v>
       </c>
     </row>
     <row r="15">
@@ -20305,7 +20307,7 @@
         </is>
       </c>
       <c r="D9" s="477" t="n">
-        <v>374</v>
+        <v>370.64</v>
       </c>
       <c r="E9" s="36" t="n">
         <v>2801644.86</v>
@@ -20346,7 +20348,7 @@
         </is>
       </c>
       <c r="D10" s="477" t="n">
-        <v>291.89</v>
+        <v>288.41</v>
       </c>
       <c r="E10" s="36" t="n">
         <v>3438605.5</v>
@@ -20387,7 +20389,7 @@
         </is>
       </c>
       <c r="D11" s="477" t="n">
-        <v>599.8200000000001</v>
+        <v>597.25</v>
       </c>
       <c r="E11" s="36" t="n">
         <v>1503313</v>
@@ -20428,7 +20430,7 @@
         </is>
       </c>
       <c r="D12" s="477" t="n">
-        <v>20.68</v>
+        <v>20.64</v>
       </c>
       <c r="E12" s="36" t="n">
         <v>49113.28</v>

</xml_diff>

<commit_message>
fix(pdf): legende p5 sous les barres + donut p7 fallback secteur si peers sans ticker
Page 5 — Marge chart : legende deplacee sous l'axe X (bbox_to_anchor, ncol=3)
pour eliminer le chevauchement avec les annotations de valeurs sur les barres.

Page 7 — Donut sectoriel : ajout fallback par secteur quand la synthese LLM
ne fournit pas de ticker dans comparable_peers. Mapping pour 11 secteurs
(consumer cyclical, technology, health, financ, energy, etc.) — TSLA affiche
desormais 95% du secteur Consumer Cyclical vs GM/F/RIVN/LCID/XPEV.

Previews AAPL et TSLA mis a jour.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/preview/AAPL/AAPL_financials.xlsx
+++ b/preview/AAPL/AAPL_financials.xlsx
@@ -9431,7 +9431,7 @@
       <c r="F95" s="266" t="n"/>
       <c r="G95" s="266" t="n"/>
       <c r="H95" s="266" t="n">
-        <v>254.2</v>
+        <v>253.53</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -9557,7 +9557,7 @@
       <c r="F100" s="266" t="n"/>
       <c r="G100" s="266" t="n"/>
       <c r="H100" s="266" t="n">
-        <v>0.0432</v>
+        <v>0.0433</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -9625,7 +9625,7 @@
       <c r="F103" s="266" t="n"/>
       <c r="G103" s="266" t="n"/>
       <c r="H103" s="266" t="n">
-        <v>0.0582</v>
+        <v>0.0583</v>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
@@ -10109,7 +10109,7 @@
       <c r="B130" s="51" t="n"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Apple maintient une position dominante dans les services et l'innovation hardware malgré des défis macroéconomiques. La valorisation reste attractive avec une marge nette de 26.9% et un ROIC de 84.4%.</t>
+          <t>Apple maintient une croissance solide avec des marges élevées et une trésorerie abondante. La valorisation reste justifiée par l'innovation et l'écosystème intégré. Les risques géopolitiques et la dép</t>
         </is>
       </c>
     </row>
@@ -10117,7 +10117,7 @@
       <c r="B131" s="51" t="n"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Invalidation : Régulation App Store, récession mondiale ou échec iPhone 17</t>
+          <t>Invalidation : Récession macro, régulation IA stricte ou perte de parts de marché en Chine</t>
         </is>
       </c>
     </row>
@@ -10412,7 +10412,7 @@
         </is>
       </c>
       <c r="C14" s="536" t="n">
-        <v>254.2</v>
+        <v>253.53</v>
       </c>
     </row>
     <row r="15">
@@ -20307,7 +20307,7 @@
         </is>
       </c>
       <c r="D9" s="477" t="n">
-        <v>370.64</v>
+        <v>370.18</v>
       </c>
       <c r="E9" s="36" t="n">
         <v>2801644.86</v>
@@ -20348,7 +20348,7 @@
         </is>
       </c>
       <c r="D10" s="477" t="n">
-        <v>288.41</v>
+        <v>288.09</v>
       </c>
       <c r="E10" s="36" t="n">
         <v>3438605.5</v>
@@ -20389,7 +20389,7 @@
         </is>
       </c>
       <c r="D11" s="477" t="n">
-        <v>597.25</v>
+        <v>598.23</v>
       </c>
       <c r="E11" s="36" t="n">
         <v>1503313</v>
@@ -20430,7 +20430,7 @@
         </is>
       </c>
       <c r="D12" s="477" t="n">
-        <v>20.64</v>
+        <v>20.61</v>
       </c>
       <c r="E12" s="36" t="n">
         <v>49113.28</v>

</xml_diff>

<commit_message>
fix(pdf): 4 correctifs visuels AAPL — marges peers, donut devise, risques cover, barres
P1 - Points cles : 'Risque 1/2' -> fallback sur synthesis.negative_themes
     quand devil.counter_risks est vide (Apple: regulation App Store, concurrence IA)

P5 - Bars chart : figsize 2.5->3.2, fontsize 9->8, clip_on=False
     pour eviter la troncature des labels sur barres de hauteurs proches

P6 - Comparables marges : _norm_margin() normalise les valeurs LLM
     (LLM retourne parfois gross_margin=68 au lieu de 0.68 -> affichait 6800%)
     Corrige SANS toucher _frpct (evite la regression ROE=151% -> 1.5%)

P7 - Donut sectoriel : filtrage devise dans _fetch_pie_data
     Skip les tickers non-USD (ex: 605930.KS Samsung KRW -> affichait 98%)
     Apple: AAPL 27% / GOOGL 25% / MSFT 20% / AMZN 17% / META 11%

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/preview/AAPL/AAPL_financials.xlsx
+++ b/preview/AAPL/AAPL_financials.xlsx
@@ -9431,7 +9431,7 @@
       <c r="F95" s="266" t="n"/>
       <c r="G95" s="266" t="n"/>
       <c r="H95" s="266" t="n">
-        <v>253.53</v>
+        <v>253.03</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -9557,7 +9557,7 @@
       <c r="F100" s="266" t="n"/>
       <c r="G100" s="266" t="n"/>
       <c r="H100" s="266" t="n">
-        <v>0.0433</v>
+        <v>0.0432</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -9625,7 +9625,7 @@
       <c r="F103" s="266" t="n"/>
       <c r="G103" s="266" t="n"/>
       <c r="H103" s="266" t="n">
-        <v>0.0583</v>
+        <v>0.0582</v>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
@@ -9693,7 +9693,7 @@
       <c r="F106" s="266" t="n"/>
       <c r="G106" s="266" t="n"/>
       <c r="H106" s="266" t="n">
-        <v>0.9742</v>
+        <v>0.9741</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1">
@@ -9713,7 +9713,7 @@
       <c r="F107" s="266" t="n"/>
       <c r="G107" s="266" t="n"/>
       <c r="H107" s="266" t="n">
-        <v>0.0258</v>
+        <v>0.0259</v>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1">
@@ -10071,7 +10071,7 @@
       <c r="B127" s="51" t="n"/>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Cible Base : 285.0</t>
+          <t>Cible Base : 275.0</t>
         </is>
       </c>
     </row>
@@ -10101,7 +10101,7 @@
       <c r="B129" s="51" t="n"/>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Cible Bear : 240.0</t>
+          <t>Cible Bear : 220.0</t>
         </is>
       </c>
     </row>
@@ -10109,7 +10109,7 @@
       <c r="B130" s="51" t="n"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Apple maintient une croissance solide avec des marges élevées et une trésorerie abondante. La valorisation reste justifiée par l'innovation et l'écosystème intégré. Les risques géopolitiques et la dép</t>
+          <t>Apple affiche une croissance résiliente avec des marges robustes et une trésorerie abondante. Le cours actuel sous-évalue le potentiel de l'IA intégrée et des services récurrents. La valorisation rest</t>
         </is>
       </c>
     </row>
@@ -10117,7 +10117,7 @@
       <c r="B131" s="51" t="n"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Invalidation : Récession macro, régulation IA stricte ou perte de parts de marché en Chine</t>
+          <t>Invalidation : Récession macro, régulation IA stricte ou échec produit iPhone 16</t>
         </is>
       </c>
     </row>
@@ -10412,7 +10412,7 @@
         </is>
       </c>
       <c r="C14" s="536" t="n">
-        <v>253.53</v>
+        <v>253.02</v>
       </c>
     </row>
     <row r="15">
@@ -20307,7 +20307,7 @@
         </is>
       </c>
       <c r="D9" s="477" t="n">
-        <v>370.18</v>
+        <v>369.73</v>
       </c>
       <c r="E9" s="36" t="n">
         <v>2801644.86</v>
@@ -20348,7 +20348,7 @@
         </is>
       </c>
       <c r="D10" s="477" t="n">
-        <v>288.09</v>
+        <v>287.52</v>
       </c>
       <c r="E10" s="36" t="n">
         <v>3438605.5</v>
@@ -20389,7 +20389,7 @@
         </is>
       </c>
       <c r="D11" s="477" t="n">
-        <v>598.23</v>
+        <v>595.45</v>
       </c>
       <c r="E11" s="36" t="n">
         <v>1503313</v>
@@ -20430,7 +20430,7 @@
         </is>
       </c>
       <c r="D12" s="477" t="n">
-        <v>20.61</v>
+        <v>20.57</v>
       </c>
       <c r="E12" s="36" t="n">
         <v>49113.28</v>

</xml_diff>

<commit_message>
chore(preview): AAPL outputs regeneres
</commit_message>
<xml_diff>
--- a/preview/AAPL/AAPL_financials.xlsx
+++ b/preview/AAPL/AAPL_financials.xlsx
@@ -9985,7 +9985,7 @@
       </c>
       <c r="D120" s="272" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="E120" s="273" t="n"/>
@@ -20427,7 +20427,7 @@
         <v>356.77</v>
       </c>
       <c r="E9" s="36" t="n">
-        <v>2751373.51</v>
+        <v>2683057.73</v>
       </c>
       <c r="F9" s="36" t="n">
         <v>305453.01</v>
@@ -20445,7 +20445,7 @@
       </c>
       <c r="J9" s="479" t="n"/>
       <c r="K9" s="477" t="n">
-        <v>15.99</v>
+        <v>15.98</v>
       </c>
       <c r="L9" s="478">
         <f>IFERROR(D9/K9,"–")</f>
@@ -20468,7 +20468,7 @@
         <v>273.76</v>
       </c>
       <c r="E10" s="36" t="n">
-        <v>3336264.74</v>
+        <v>3251827.64</v>
       </c>
       <c r="F10" s="36" t="n">
         <v>402836</v>
@@ -20509,7 +20509,7 @@
         <v>525.72</v>
       </c>
       <c r="E11" s="36" t="n">
-        <v>1388521.85</v>
+        <v>1333326.91</v>
       </c>
       <c r="F11" s="36" t="n">
         <v>200966</v>
@@ -20527,7 +20527,7 @@
       </c>
       <c r="J11" s="479" t="n"/>
       <c r="K11" s="477" t="n">
-        <v>23.49</v>
+        <v>23.5</v>
       </c>
       <c r="L11" s="478">
         <f>IFERROR(D11/K11,"–")</f>
@@ -20550,7 +20550,7 @@
         <v>19.91</v>
       </c>
       <c r="E12" s="36" t="n">
-        <v>45890.52</v>
+        <v>45174.36</v>
       </c>
       <c r="F12" s="36" t="n">
         <v>13170287.58</v>

</xml_diff>